<commit_message>
[UPDATE] - Baixando anexo do email. OK
</commit_message>
<xml_diff>
--- a/Cube_finish.xlsx
+++ b/Cube_finish.xlsx
@@ -503,26 +503,18 @@
           <t>Pads Zone A / Core A</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>10/03/2022</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2360</t>
-        </is>
+      <c r="E2" s="2" t="n">
+        <v>44456</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2380</v>
       </c>
       <c r="G2" t="n">
         <v>32.8</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>52.7</t>
-        </is>
-      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>40N</t>
@@ -548,22 +540,16 @@
           <t>Pads Zone A / Core A</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>09/03/2022</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2400</t>
-        </is>
+      <c r="E3" s="2" t="n">
+        <v>44477</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2380</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>51.0</t>
-        </is>
+      <c r="I3" t="n">
+        <v>44.2</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
@@ -591,22 +577,16 @@
           <t>Pads Zone A / Core A</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>09/03/2022</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2430</t>
-        </is>
+      <c r="E4" s="2" t="n">
+        <v>44463</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2420</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>50.1</t>
-        </is>
+      <c r="I4" t="n">
+        <v>33.5</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
@@ -634,20 +614,14 @@
           <t>Pads Zone A / Core A</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>09/03/2022</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2390</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>52.7(6Days)</t>
-        </is>
+      <c r="E5" s="2" t="n">
+        <v>44456</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G5" t="n">
+        <v>30.2</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -677,22 +651,16 @@
           <t>Pads Zone A / Core A</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>10/03/2022</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2380</t>
-        </is>
+      <c r="E6" s="2" t="n">
+        <v>44477</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2360</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>45.5</t>
-        </is>
+      <c r="I6" t="n">
+        <v>42.2</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
@@ -720,22 +688,16 @@
           <t>Pads Zone A / Core A</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>10/03/2022</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2380</t>
-        </is>
+      <c r="E7" s="2" t="n">
+        <v>44477</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2360</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>39.3</t>
-        </is>
+      <c r="I7" t="n">
+        <v>42</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
@@ -1061,15 +1023,11 @@
           <t>Mainholes</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>10/03/2022</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>2360</t>
-        </is>
+      <c r="E16" s="2" t="n">
+        <v>44454</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2400</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1078,11 +1036,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>52.7</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>40N</t>
@@ -1108,25 +1062,17 @@
           <t>Mainholes</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>09/03/2022</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>2400</t>
-        </is>
+      <c r="E17" s="2" t="n">
+        <v>44463</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2400</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
         <v>33.8</v>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>51.0</t>
-        </is>
-      </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
@@ -1153,25 +1099,17 @@
           <t>Mainholes</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>09/03/2022</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>2430</t>
-        </is>
+      <c r="E18" s="2" t="n">
+        <v>44463</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2420</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
         <v>33.5</v>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>50.1</t>
-        </is>
-      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
@@ -1198,21 +1136,13 @@
           <t>Mainholes</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>09/03/2022</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>2390</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>52.7(6Days)</t>
-        </is>
-      </c>
+      <c r="E19" s="2" t="n">
+        <v>44491</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="n">
@@ -17286,15 +17216,19 @@
           <t>First Floor Wall (30-45)(B-Z)</t>
         </is>
       </c>
-      <c r="E463" s="2" t="n">
-        <v>44601</v>
-      </c>
-      <c r="F463" t="n">
-        <v>2370</v>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>09/02/2022</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>2370</t>
+        </is>
       </c>
       <c r="G463" t="inlineStr">
         <is>
-          <t>9 Days(33.9)</t>
+          <t>33.9(9Days)</t>
         </is>
       </c>
       <c r="H463" t="inlineStr"/>
@@ -17402,15 +17336,19 @@
           <t>Second Floor Slab - Area 1</t>
         </is>
       </c>
-      <c r="E467" s="2" t="n">
-        <v>44601</v>
-      </c>
-      <c r="F467" t="n">
-        <v>2340</v>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>09/02/2022</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
       </c>
       <c r="G467" t="inlineStr">
         <is>
-          <t>9 Days(38.4)</t>
+          <t>38.4(9Days)</t>
         </is>
       </c>
       <c r="H467" t="inlineStr"/>
@@ -17437,15 +17375,19 @@
           <t>Second Floor Slab - Area 1</t>
         </is>
       </c>
-      <c r="E468" s="2" t="n">
-        <v>44601</v>
-      </c>
-      <c r="F468" t="n">
-        <v>2340</v>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>09/02/2022</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
       </c>
       <c r="G468" t="inlineStr">
         <is>
-          <t>9 Days(37.7)</t>
+          <t>37.7(9Days)</t>
         </is>
       </c>
       <c r="H468" t="inlineStr"/>
@@ -17553,14 +17495,20 @@
           <t>First Floor Walls (31-37)(G-DD)</t>
         </is>
       </c>
-      <c r="E472" s="2" t="n">
-        <v>44601</v>
-      </c>
-      <c r="F472" t="n">
-        <v>2300</v>
-      </c>
-      <c r="G472" t="n">
-        <v>32.7</v>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>09/02/2022</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>2300</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>32.7</t>
+        </is>
       </c>
       <c r="H472" t="inlineStr"/>
       <c r="I472" t="inlineStr"/>

</xml_diff>

<commit_message>
[UPDATE] - Funcionando todo os passos. OK
</commit_message>
<xml_diff>
--- a/Cube_finish.xlsx
+++ b/Cube_finish.xlsx
@@ -13519,12 +13519,24 @@
           <t>First Floor W1 (DD-KK) (8-9)</t>
         </is>
       </c>
-      <c r="D409" s="2" t="inlineStr"/>
-      <c r="E409" s="2" t="inlineStr"/>
+      <c r="D409" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2022</t>
+        </is>
+      </c>
+      <c r="E409" s="2" t="inlineStr">
+        <is>
+          <t>2390</t>
+        </is>
+      </c>
       <c r="F409" s="2" t="inlineStr"/>
       <c r="G409" s="2" t="inlineStr"/>
       <c r="H409" s="2" t="inlineStr"/>
-      <c r="I409" s="2" t="inlineStr"/>
+      <c r="I409" s="2" t="inlineStr">
+        <is>
+          <t>52.7</t>
+        </is>
+      </c>
       <c r="J409" s="2" t="inlineStr">
         <is>
           <t>37N</t>
@@ -13634,8 +13646,10 @@
           <t>10/03/2022</t>
         </is>
       </c>
-      <c r="E413" s="2" t="n">
-        <v>2360</v>
+      <c r="E413" s="2" t="inlineStr">
+        <is>
+          <t>2360</t>
+        </is>
       </c>
       <c r="F413" s="2" t="inlineStr"/>
       <c r="G413" s="2" t="inlineStr"/>
@@ -13750,8 +13764,10 @@
           <t>11/03/2022</t>
         </is>
       </c>
-      <c r="E417" s="2" t="n">
-        <v>2350</v>
+      <c r="E417" s="2" t="inlineStr">
+        <is>
+          <t>2350</t>
+        </is>
       </c>
       <c r="F417" s="2" t="inlineStr"/>
       <c r="G417" s="2" t="inlineStr"/>
@@ -13868,8 +13884,10 @@
           <t>14/03/2022</t>
         </is>
       </c>
-      <c r="E421" s="2" t="n">
-        <v>2380</v>
+      <c r="E421" s="2" t="inlineStr">
+        <is>
+          <t>2380</t>
+        </is>
       </c>
       <c r="F421" s="2" t="inlineStr"/>
       <c r="G421" s="2" t="inlineStr"/>
@@ -13980,8 +13998,10 @@
           <t>14/03/2022</t>
         </is>
       </c>
-      <c r="E425" s="2" t="n">
-        <v>2370</v>
+      <c r="E425" s="2" t="inlineStr">
+        <is>
+          <t>2370</t>
+        </is>
       </c>
       <c r="F425" s="2" t="inlineStr"/>
       <c r="G425" s="2" t="inlineStr"/>
@@ -14182,8 +14202,10 @@
           <t>16/03/2022</t>
         </is>
       </c>
-      <c r="E432" s="2" t="n">
-        <v>2380</v>
+      <c r="E432" s="2" t="inlineStr">
+        <is>
+          <t>2380</t>
+        </is>
       </c>
       <c r="F432" s="2" t="inlineStr"/>
       <c r="G432" s="2" t="inlineStr"/>
@@ -14326,8 +14348,10 @@
           <t>17/03/2022</t>
         </is>
       </c>
-      <c r="E437" s="2" t="n">
-        <v>2360</v>
+      <c r="E437" s="2" t="inlineStr">
+        <is>
+          <t>2360</t>
+        </is>
       </c>
       <c r="F437" s="2" t="inlineStr"/>
       <c r="G437" s="2" t="inlineStr"/>
@@ -14358,8 +14382,10 @@
           <t>17/03/2022</t>
         </is>
       </c>
-      <c r="E438" s="2" t="n">
-        <v>2330</v>
+      <c r="E438" s="2" t="inlineStr">
+        <is>
+          <t>2330</t>
+        </is>
       </c>
       <c r="F438" s="2" t="inlineStr"/>
       <c r="G438" s="2" t="inlineStr"/>
@@ -14474,8 +14500,10 @@
           <t>18/03/2022</t>
         </is>
       </c>
-      <c r="E442" s="2" t="n">
-        <v>2420</v>
+      <c r="E442" s="2" t="inlineStr">
+        <is>
+          <t>2420</t>
+        </is>
       </c>
       <c r="F442" s="2" t="inlineStr"/>
       <c r="G442" s="2" t="inlineStr"/>
@@ -14592,8 +14620,10 @@
           <t>21/03/2022</t>
         </is>
       </c>
-      <c r="E446" s="2" t="n">
-        <v>2370</v>
+      <c r="E446" s="2" t="inlineStr">
+        <is>
+          <t>2370</t>
+        </is>
       </c>
       <c r="F446" s="2" t="inlineStr"/>
       <c r="G446" s="2" t="inlineStr"/>
@@ -14811,12 +14841,24 @@
           <t>First Floor Walls (22-35)(U-GG)</t>
         </is>
       </c>
-      <c r="D454" s="2" t="inlineStr"/>
-      <c r="E454" s="2" t="inlineStr"/>
+      <c r="D454" s="2" t="inlineStr">
+        <is>
+          <t>23/03/2022</t>
+        </is>
+      </c>
+      <c r="E454" s="2" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
       <c r="F454" s="2" t="inlineStr"/>
       <c r="G454" s="2" t="inlineStr"/>
       <c r="H454" s="2" t="inlineStr"/>
-      <c r="I454" s="2" t="inlineStr"/>
+      <c r="I454" s="2" t="inlineStr">
+        <is>
+          <t>46.8</t>
+        </is>
+      </c>
       <c r="J454" s="2" t="inlineStr"/>
     </row>
     <row r="455">
@@ -15966,13 +16008,17 @@
           <t>09/03/2022</t>
         </is>
       </c>
-      <c r="E498" s="2" t="n">
-        <v>2400</v>
+      <c r="E498" s="2" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
       </c>
       <c r="F498" s="2" t="inlineStr"/>
       <c r="G498" s="2" t="inlineStr"/>
-      <c r="H498" s="2" t="n">
-        <v>51</v>
+      <c r="H498" s="2" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
       </c>
       <c r="I498" s="2" t="inlineStr"/>
       <c r="J498" s="2" t="inlineStr"/>
@@ -15997,13 +16043,17 @@
           <t>09/03/2022</t>
         </is>
       </c>
-      <c r="E499" s="2" t="n">
-        <v>2430</v>
+      <c r="E499" s="2" t="inlineStr">
+        <is>
+          <t>2430</t>
+        </is>
       </c>
       <c r="F499" s="2" t="inlineStr"/>
       <c r="G499" s="2" t="inlineStr"/>
-      <c r="H499" s="2" t="n">
-        <v>50.1</v>
+      <c r="H499" s="2" t="inlineStr">
+        <is>
+          <t>50.1</t>
+        </is>
       </c>
       <c r="I499" s="2" t="inlineStr"/>
       <c r="J499" s="2" t="inlineStr"/>
@@ -16078,13 +16128,17 @@
           <t>10/03/2022</t>
         </is>
       </c>
-      <c r="E502" s="2" t="n">
-        <v>2380</v>
+      <c r="E502" s="2" t="inlineStr">
+        <is>
+          <t>2380</t>
+        </is>
       </c>
       <c r="F502" s="2" t="inlineStr"/>
       <c r="G502" s="2" t="inlineStr"/>
-      <c r="H502" s="2" t="n">
-        <v>45.5</v>
+      <c r="H502" s="2" t="inlineStr">
+        <is>
+          <t>45.5</t>
+        </is>
       </c>
       <c r="I502" s="2" t="inlineStr"/>
       <c r="J502" s="2" t="inlineStr"/>
@@ -16108,13 +16162,17 @@
           <t>10/03/2022</t>
         </is>
       </c>
-      <c r="E503" s="2" t="n">
-        <v>2380</v>
+      <c r="E503" s="2" t="inlineStr">
+        <is>
+          <t>2380</t>
+        </is>
       </c>
       <c r="F503" s="2" t="inlineStr"/>
       <c r="G503" s="2" t="inlineStr"/>
-      <c r="H503" s="2" t="n">
-        <v>39.3</v>
+      <c r="H503" s="2" t="inlineStr">
+        <is>
+          <t>39.3</t>
+        </is>
       </c>
       <c r="I503" s="2" t="inlineStr"/>
       <c r="J503" s="2" t="inlineStr"/>
@@ -16216,13 +16274,17 @@
           <t>11/03/2022</t>
         </is>
       </c>
-      <c r="E507" s="2" t="n">
-        <v>2360</v>
+      <c r="E507" s="2" t="inlineStr">
+        <is>
+          <t>2360</t>
+        </is>
       </c>
       <c r="F507" s="2" t="inlineStr"/>
       <c r="G507" s="2" t="inlineStr"/>
-      <c r="H507" s="2" t="n">
-        <v>43</v>
+      <c r="H507" s="2" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
       </c>
       <c r="I507" s="2" t="inlineStr"/>
       <c r="J507" s="2" t="inlineStr"/>
@@ -16246,13 +16308,17 @@
           <t>11/03/2022</t>
         </is>
       </c>
-      <c r="E508" s="2" t="n">
-        <v>2370</v>
+      <c r="E508" s="2" t="inlineStr">
+        <is>
+          <t>2370</t>
+        </is>
       </c>
       <c r="F508" s="2" t="inlineStr"/>
       <c r="G508" s="2" t="inlineStr"/>
-      <c r="H508" s="2" t="n">
-        <v>44.5</v>
+      <c r="H508" s="2" t="inlineStr">
+        <is>
+          <t>44.5</t>
+        </is>
       </c>
       <c r="I508" s="2" t="inlineStr"/>
       <c r="J508" s="2" t="inlineStr"/>
@@ -16326,13 +16392,17 @@
           <t>14/03/2022</t>
         </is>
       </c>
-      <c r="E511" s="2" t="n">
-        <v>2330</v>
+      <c r="E511" s="2" t="inlineStr">
+        <is>
+          <t>2330</t>
+        </is>
       </c>
       <c r="F511" s="2" t="inlineStr"/>
       <c r="G511" s="2" t="inlineStr"/>
-      <c r="H511" s="2" t="n">
-        <v>39.6</v>
+      <c r="H511" s="2" t="inlineStr">
+        <is>
+          <t>39.6</t>
+        </is>
       </c>
       <c r="I511" s="2" t="inlineStr"/>
       <c r="J511" s="2" t="inlineStr"/>
@@ -16356,13 +16426,17 @@
           <t>14/03/2022</t>
         </is>
       </c>
-      <c r="E512" s="2" t="n">
-        <v>2330</v>
+      <c r="E512" s="2" t="inlineStr">
+        <is>
+          <t>2330</t>
+        </is>
       </c>
       <c r="F512" s="2" t="inlineStr"/>
       <c r="G512" s="2" t="inlineStr"/>
-      <c r="H512" s="2" t="n">
-        <v>39</v>
+      <c r="H512" s="2" t="inlineStr">
+        <is>
+          <t>39.0</t>
+        </is>
       </c>
       <c r="I512" s="2" t="inlineStr"/>
       <c r="J512" s="2" t="inlineStr"/>
@@ -16430,13 +16504,17 @@
           <t>14/03/2022</t>
         </is>
       </c>
-      <c r="E515" s="2" t="n">
-        <v>2380</v>
+      <c r="E515" s="2" t="inlineStr">
+        <is>
+          <t>2380</t>
+        </is>
       </c>
       <c r="F515" s="2" t="inlineStr"/>
       <c r="G515" s="2" t="inlineStr"/>
-      <c r="H515" s="2" t="n">
-        <v>52.9</v>
+      <c r="H515" s="2" t="inlineStr">
+        <is>
+          <t>52.9</t>
+        </is>
       </c>
       <c r="I515" s="2" t="inlineStr"/>
       <c r="J515" s="2" t="inlineStr"/>
@@ -16460,13 +16538,17 @@
           <t>14/03/2022</t>
         </is>
       </c>
-      <c r="E516" s="2" t="n">
-        <v>2380</v>
+      <c r="E516" s="2" t="inlineStr">
+        <is>
+          <t>2380</t>
+        </is>
       </c>
       <c r="F516" s="2" t="inlineStr"/>
       <c r="G516" s="2" t="inlineStr"/>
-      <c r="H516" s="2" t="n">
-        <v>51.8</v>
+      <c r="H516" s="2" t="inlineStr">
+        <is>
+          <t>51.8</t>
+        </is>
       </c>
       <c r="I516" s="2" t="inlineStr"/>
       <c r="J516" s="2" t="inlineStr"/>
@@ -16512,8 +16594,10 @@
           <t>09/03/2022</t>
         </is>
       </c>
-      <c r="E518" s="2" t="n">
-        <v>2360</v>
+      <c r="E518" s="2" t="inlineStr">
+        <is>
+          <t>2360</t>
+        </is>
       </c>
       <c r="F518" s="2" t="inlineStr">
         <is>
@@ -16544,13 +16628,17 @@
           <t>15/03/2022</t>
         </is>
       </c>
-      <c r="E519" s="2" t="n">
-        <v>2350</v>
+      <c r="E519" s="2" t="inlineStr">
+        <is>
+          <t>2350</t>
+        </is>
       </c>
       <c r="F519" s="2" t="inlineStr"/>
       <c r="G519" s="2" t="inlineStr"/>
-      <c r="H519" s="2" t="n">
-        <v>45.6</v>
+      <c r="H519" s="2" t="inlineStr">
+        <is>
+          <t>45.6</t>
+        </is>
       </c>
       <c r="I519" s="2" t="inlineStr"/>
       <c r="J519" s="2" t="inlineStr"/>
@@ -16574,13 +16662,17 @@
           <t>15/03/2022</t>
         </is>
       </c>
-      <c r="E520" s="2" t="n">
-        <v>2360</v>
+      <c r="E520" s="2" t="inlineStr">
+        <is>
+          <t>2360</t>
+        </is>
       </c>
       <c r="F520" s="2" t="inlineStr"/>
       <c r="G520" s="2" t="inlineStr"/>
-      <c r="H520" s="2" t="n">
-        <v>41.9</v>
+      <c r="H520" s="2" t="inlineStr">
+        <is>
+          <t>41.9</t>
+        </is>
       </c>
       <c r="I520" s="2" t="inlineStr"/>
       <c r="J520" s="2" t="inlineStr"/>
@@ -16626,8 +16718,10 @@
           <t>09/03/2022</t>
         </is>
       </c>
-      <c r="E522" s="2" t="n">
-        <v>2380</v>
+      <c r="E522" s="2" t="inlineStr">
+        <is>
+          <t>2380</t>
+        </is>
       </c>
       <c r="F522" s="2" t="inlineStr">
         <is>
@@ -16658,13 +16752,17 @@
           <t>16/03/2022</t>
         </is>
       </c>
-      <c r="E523" s="2" t="n">
-        <v>2370</v>
+      <c r="E523" s="2" t="inlineStr">
+        <is>
+          <t>2370</t>
+        </is>
       </c>
       <c r="F523" s="2" t="inlineStr"/>
       <c r="G523" s="2" t="inlineStr"/>
-      <c r="H523" s="2" t="n">
-        <v>50.4</v>
+      <c r="H523" s="2" t="inlineStr">
+        <is>
+          <t>50.4</t>
+        </is>
       </c>
       <c r="I523" s="2" t="inlineStr"/>
       <c r="J523" s="2" t="inlineStr"/>
@@ -16688,13 +16786,17 @@
           <t>16/03/2022</t>
         </is>
       </c>
-      <c r="E524" s="2" t="n">
-        <v>2370</v>
+      <c r="E524" s="2" t="inlineStr">
+        <is>
+          <t>2370</t>
+        </is>
       </c>
       <c r="F524" s="2" t="inlineStr"/>
       <c r="G524" s="2" t="inlineStr"/>
-      <c r="H524" s="2" t="n">
-        <v>49.7</v>
+      <c r="H524" s="2" t="inlineStr">
+        <is>
+          <t>49.7</t>
+        </is>
       </c>
       <c r="I524" s="2" t="inlineStr"/>
       <c r="J524" s="2" t="inlineStr"/>
@@ -16740,8 +16842,10 @@
           <t>09/03/2022</t>
         </is>
       </c>
-      <c r="E526" s="2" t="n">
-        <v>2380</v>
+      <c r="E526" s="2" t="inlineStr">
+        <is>
+          <t>2380</t>
+        </is>
       </c>
       <c r="F526" s="2" t="inlineStr">
         <is>
@@ -16772,13 +16876,17 @@
           <t>17/03/2022</t>
         </is>
       </c>
-      <c r="E527" s="2" t="n">
-        <v>2380</v>
+      <c r="E527" s="2" t="inlineStr">
+        <is>
+          <t>2380</t>
+        </is>
       </c>
       <c r="F527" s="2" t="inlineStr"/>
       <c r="G527" s="2" t="inlineStr"/>
-      <c r="H527" s="2" t="n">
-        <v>49.7</v>
+      <c r="H527" s="2" t="inlineStr">
+        <is>
+          <t>49.7</t>
+        </is>
       </c>
       <c r="I527" s="2" t="inlineStr"/>
       <c r="J527" s="2" t="inlineStr"/>
@@ -16802,13 +16910,17 @@
           <t>17/03/2022</t>
         </is>
       </c>
-      <c r="E528" s="2" t="n">
-        <v>2390</v>
+      <c r="E528" s="2" t="inlineStr">
+        <is>
+          <t>2390</t>
+        </is>
       </c>
       <c r="F528" s="2" t="inlineStr"/>
       <c r="G528" s="2" t="inlineStr"/>
-      <c r="H528" s="2" t="n">
-        <v>48.6</v>
+      <c r="H528" s="2" t="inlineStr">
+        <is>
+          <t>48.6</t>
+        </is>
       </c>
       <c r="I528" s="2" t="inlineStr"/>
       <c r="J528" s="2" t="inlineStr"/>
@@ -16854,8 +16966,10 @@
           <t>09/03/2022</t>
         </is>
       </c>
-      <c r="E530" s="2" t="n">
-        <v>2380</v>
+      <c r="E530" s="2" t="inlineStr">
+        <is>
+          <t>2380</t>
+        </is>
       </c>
       <c r="F530" s="2" t="inlineStr">
         <is>
@@ -16886,13 +17000,17 @@
           <t>18/03/2022</t>
         </is>
       </c>
-      <c r="E531" s="2" t="n">
-        <v>2390</v>
+      <c r="E531" s="2" t="inlineStr">
+        <is>
+          <t>2390</t>
+        </is>
       </c>
       <c r="F531" s="2" t="inlineStr"/>
       <c r="G531" s="2" t="inlineStr"/>
-      <c r="H531" s="2" t="n">
-        <v>45.6</v>
+      <c r="H531" s="2" t="inlineStr">
+        <is>
+          <t>45.6</t>
+        </is>
       </c>
       <c r="I531" s="2" t="inlineStr"/>
       <c r="J531" s="2" t="inlineStr"/>
@@ -16916,13 +17034,17 @@
           <t>18/03/2022</t>
         </is>
       </c>
-      <c r="E532" s="2" t="n">
-        <v>2400</v>
+      <c r="E532" s="2" t="inlineStr">
+        <is>
+          <t>2400</t>
+        </is>
       </c>
       <c r="F532" s="2" t="inlineStr"/>
       <c r="G532" s="2" t="inlineStr"/>
-      <c r="H532" s="2" t="n">
-        <v>46.8</v>
+      <c r="H532" s="2" t="inlineStr">
+        <is>
+          <t>46.8</t>
+        </is>
       </c>
       <c r="I532" s="2" t="inlineStr"/>
       <c r="J532" s="2" t="inlineStr"/>
@@ -17002,13 +17124,17 @@
           <t>21/03/2022</t>
         </is>
       </c>
-      <c r="E535" s="2" t="n">
-        <v>2370</v>
+      <c r="E535" s="2" t="inlineStr">
+        <is>
+          <t>2370</t>
+        </is>
       </c>
       <c r="F535" s="2" t="inlineStr"/>
       <c r="G535" s="2" t="inlineStr"/>
-      <c r="H535" s="2" t="n">
-        <v>44.4</v>
+      <c r="H535" s="2" t="inlineStr">
+        <is>
+          <t>44.4</t>
+        </is>
       </c>
       <c r="I535" s="2" t="inlineStr"/>
       <c r="J535" s="2" t="inlineStr"/>
@@ -17032,13 +17158,17 @@
           <t>21/03/2022</t>
         </is>
       </c>
-      <c r="E536" s="2" t="n">
-        <v>2360</v>
+      <c r="E536" s="2" t="inlineStr">
+        <is>
+          <t>2360</t>
+        </is>
       </c>
       <c r="F536" s="2" t="inlineStr"/>
       <c r="G536" s="2" t="inlineStr"/>
-      <c r="H536" s="2" t="n">
-        <v>45.3</v>
+      <c r="H536" s="2" t="inlineStr">
+        <is>
+          <t>45.3</t>
+        </is>
       </c>
       <c r="I536" s="2" t="inlineStr"/>
       <c r="J536" s="2" t="inlineStr"/>
@@ -17361,11 +17491,23 @@
           <t>2nd Floor Walls (A-E)(35-45),W1(U-GG)(31-35),W1 (Z-EE)(37-41)</t>
         </is>
       </c>
-      <c r="D547" s="2" t="inlineStr"/>
-      <c r="E547" s="2" t="inlineStr"/>
+      <c r="D547" s="2" t="inlineStr">
+        <is>
+          <t>23/03/2022</t>
+        </is>
+      </c>
+      <c r="E547" s="2" t="inlineStr">
+        <is>
+          <t>2390</t>
+        </is>
+      </c>
       <c r="F547" s="2" t="inlineStr"/>
       <c r="G547" s="2" t="inlineStr"/>
-      <c r="H547" s="2" t="inlineStr"/>
+      <c r="H547" s="2" t="inlineStr">
+        <is>
+          <t>40.2</t>
+        </is>
+      </c>
       <c r="I547" s="2" t="inlineStr"/>
       <c r="J547" s="2" t="inlineStr"/>
     </row>
@@ -17383,11 +17525,23 @@
           <t>2nd Floor Walls (A-E)(35-45),W1(U-GG)(31-35),W1 (Z-EE)(37-41)</t>
         </is>
       </c>
-      <c r="D548" s="2" t="inlineStr"/>
-      <c r="E548" s="2" t="inlineStr"/>
+      <c r="D548" s="2" t="inlineStr">
+        <is>
+          <t>23/03/2022</t>
+        </is>
+      </c>
+      <c r="E548" s="2" t="inlineStr">
+        <is>
+          <t>2410</t>
+        </is>
+      </c>
       <c r="F548" s="2" t="inlineStr"/>
       <c r="G548" s="2" t="inlineStr"/>
-      <c r="H548" s="2" t="inlineStr"/>
+      <c r="H548" s="2" t="inlineStr">
+        <is>
+          <t>44.6</t>
+        </is>
+      </c>
       <c r="I548" s="2" t="inlineStr"/>
       <c r="J548" s="2" t="inlineStr"/>
     </row>
@@ -17432,8 +17586,10 @@
           <t>09/03/2022</t>
         </is>
       </c>
-      <c r="E550" s="2" t="n">
-        <v>2350</v>
+      <c r="E550" s="2" t="inlineStr">
+        <is>
+          <t>2350</t>
+        </is>
       </c>
       <c r="F550" s="2" t="inlineStr">
         <is>
@@ -17486,13 +17642,17 @@
           <t>14/03/2022</t>
         </is>
       </c>
-      <c r="E552" s="2" t="n">
-        <v>2340</v>
+      <c r="E552" s="2" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
       </c>
       <c r="F552" s="2" t="inlineStr"/>
       <c r="G552" s="2" t="inlineStr"/>
-      <c r="H552" s="2" t="n">
-        <v>38.2</v>
+      <c r="H552" s="2" t="inlineStr">
+        <is>
+          <t>38.2</t>
+        </is>
       </c>
       <c r="I552" s="2" t="inlineStr"/>
       <c r="J552" s="2" t="inlineStr"/>
@@ -17538,8 +17698,10 @@
           <t>11/03/2022</t>
         </is>
       </c>
-      <c r="E554" s="2" t="n">
-        <v>2320</v>
+      <c r="E554" s="2" t="inlineStr">
+        <is>
+          <t>2320</t>
+        </is>
       </c>
       <c r="F554" s="2" t="inlineStr"/>
       <c r="G554" s="2" t="inlineStr">
@@ -17636,8 +17798,10 @@
           <t>09/03/2022</t>
         </is>
       </c>
-      <c r="E558" s="2" t="n">
-        <v>2350</v>
+      <c r="E558" s="2" t="inlineStr">
+        <is>
+          <t>2350</t>
+        </is>
       </c>
       <c r="F558" s="2" t="inlineStr">
         <is>
@@ -17734,8 +17898,10 @@
           <t>09/03/2022</t>
         </is>
       </c>
-      <c r="E562" s="2" t="n">
-        <v>2370</v>
+      <c r="E562" s="2" t="inlineStr">
+        <is>
+          <t>2370</t>
+        </is>
       </c>
       <c r="F562" s="2" t="inlineStr">
         <is>
@@ -17832,8 +17998,10 @@
           <t>09/03/2022</t>
         </is>
       </c>
-      <c r="E566" s="2" t="n">
-        <v>2360</v>
+      <c r="E566" s="2" t="inlineStr">
+        <is>
+          <t>2360</t>
+        </is>
       </c>
       <c r="F566" s="2" t="inlineStr">
         <is>
@@ -17930,8 +18098,10 @@
           <t>09/03/2022</t>
         </is>
       </c>
-      <c r="E570" s="2" t="n">
-        <v>2350</v>
+      <c r="E570" s="2" t="inlineStr">
+        <is>
+          <t>2350</t>
+        </is>
       </c>
       <c r="F570" s="2" t="inlineStr">
         <is>
@@ -18028,8 +18198,10 @@
           <t>10/03/2022</t>
         </is>
       </c>
-      <c r="E574" s="2" t="n">
-        <v>2360</v>
+      <c r="E574" s="2" t="inlineStr">
+        <is>
+          <t>2360</t>
+        </is>
       </c>
       <c r="F574" s="2" t="inlineStr">
         <is>
@@ -18126,8 +18298,10 @@
           <t>11/03/2022</t>
         </is>
       </c>
-      <c r="E578" s="2" t="n">
-        <v>2380</v>
+      <c r="E578" s="2" t="inlineStr">
+        <is>
+          <t>2380</t>
+        </is>
       </c>
       <c r="F578" s="2" t="inlineStr">
         <is>

</xml_diff>